<commit_message>
📊 Horarios actualizados Línea 141 - 1832
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:09:06</t>
+          <t>Última actualización: 02:23:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:09:06</t>
+          <t>02:23:35</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:25</t>
+          <t>03:02</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,23 +498,48 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:09:06</t>
+          <t>02:23:35</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:03</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>114</v>
+        <v>85</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:23:35</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>98</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -544,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:09:06</t>
+          <t>Última actualización: 02:23:35</t>
         </is>
       </c>
     </row>
@@ -579,7 +604,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:09:06</t>
+          <t>Última actualización: 02:23:35</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1833
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:23:35</t>
+          <t>Última actualización: 03:09:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -473,17 +473,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:23:35</t>
+          <t>03:09:56</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:23:35</t>
+          <t>03:09:56</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>85</v>
+        <v>52</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,23 +523,48 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:23:35</t>
+          <t>03:09:56</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:01</t>
+          <t>04:46</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:09:56</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:53</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>104</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -556,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,14 +594,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:23:35</t>
+          <t>Última actualización: 03:09:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>03:09:56</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>04:46</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>97</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -604,7 +681,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:23:35</t>
+          <t>Última actualización: 03:09:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1834
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:09:56</t>
+          <t>Última actualización: 04:06:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:09:56</t>
+          <t>04:06:29</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:09:56</t>
+          <t>04:06:29</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:01</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:09:56</t>
+          <t>04:06:29</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:46</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>97</v>
+        <v>71</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,23 +548,98 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:09:56</t>
+          <t>04:06:29</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>104</v>
+        <v>76</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>04:06:29</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>05:47</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>101</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>04:06:29</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:49</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>103</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04:06:29</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>115</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -581,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,66 +669,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:09:56</t>
+          <t>Última actualización: 04:06:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Hora_Scrap</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Hora_Llegada</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Linea</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Minutos</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Parada</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>03:09:56</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>04:46</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>215_EL PELIGRO</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>97</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>LP1912</t>
+          <t>Total filas: 0</t>
         </is>
       </c>
     </row>
@@ -681,7 +704,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:09:56</t>
+          <t>Última actualización: 04:06:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1835
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:06:29</t>
+          <t>Última actualización: 04:46:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:06:29</t>
+          <t>04:46:10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,7 +498,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:06:29</t>
+          <t>04:46:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>47</v>
+        <v>7</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,7 +523,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:06:29</t>
+          <t>04:46:10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,7 +548,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:06:29</t>
+          <t>04:46:10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:06:29</t>
+          <t>04:46:10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>101</v>
+        <v>58</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:06:29</t>
+          <t>04:46:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:49</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:06:29</t>
+          <t>04:46:10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -637,9 +637,159 @@
         </is>
       </c>
       <c r="D12" t="n">
+        <v>75</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:46:10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:09</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>83</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:46:10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>86</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:46:10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>104</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:46:10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:34</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>108</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:46:10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>113</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:46:10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
         <v>115</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -656,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -669,14 +819,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:06:29</t>
+          <t>Última actualización: 04:46:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>04:46:10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>86</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -704,7 +906,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:06:29</t>
+          <t>Última actualización: 04:46:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1836
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:46:10</t>
+          <t>Última actualización: 05:01:37</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:34</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:34</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,14 +819,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:46:10</t>
+          <t>Última actualización: 05:01:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:46:10</t>
+          <t>05:01:37</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -874,9 +874,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:01:37</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>114</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -906,7 +931,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:46:10</t>
+          <t>Última actualización: 05:01:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1837
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:01:37</t>
+          <t>Última actualización: 05:49:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:34</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,12 +623,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:34</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,12 +723,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,23 +773,48 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>05:49:33</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>107</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -806,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,14 +844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:01:37</t>
+          <t>Última actualización: 05:49:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -860,7 +885,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -874,7 +899,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -885,7 +910,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:01:37</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -899,9 +924,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>114</v>
+        <v>66</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05:49:33</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -918,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -931,14 +981,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:01:37</t>
+          <t>Última actualización: 05:49:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>05:49:33</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>115</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1838
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:49:33</t>
+          <t>Última actualización: 06:17:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>90</v>
+        <v>42</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -708,11 +708,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>101</v>
+        <v>64</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>106</v>
+        <v>69</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,18 +803,168 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>101</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>06:17:32</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07:34</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>77</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>06:17:32</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>78</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06:17:32</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>07:36</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>107</v>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="D22" t="n">
+        <v>79</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>06:17:32</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>98</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>06:17:32</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>07:58</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>101</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>06:17:32</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>08:11</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>114</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -831,7 +981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -844,14 +994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:49:33</t>
+          <t>Última actualización: 06:17:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -910,7 +1060,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -924,7 +1074,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -935,7 +1085,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -949,9 +1099,34 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:17:32</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07:34</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>77</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -981,7 +1156,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:49:33</t>
+          <t>Última actualización: 06:17:32</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1197,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1036,7 +1211,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1839
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:17:32</t>
+          <t>Última actualización: 06:49:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>06:49</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -678,16 +678,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>06:56</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>62</v>
+        <v>7</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>62</v>
+        <v>10</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>64</v>
+        <v>30</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -778,16 +778,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>101</v>
+        <v>31</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:34</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>77</v>
+        <v>32</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -853,16 +853,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>79</v>
+        <v>40</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -928,16 +928,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>07:58</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,23 +948,348 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>46</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>46</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>06:17:32</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>79</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>48</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>66</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>06:17:32</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>07:58</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>101</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>07:59</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>70</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>06:17:32</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>08:11</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D32" t="n">
         <v>114</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>88</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>08:22</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>93</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>08:28</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>99</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>109</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>112</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>112</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -981,7 +1306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -994,14 +1319,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:17:32</t>
+          <t>Última actualización: 06:49:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1085,21 +1410,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>06:56</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>62</v>
+        <v>7</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1115,18 +1440,118 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>62</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>31</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:17:32</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>07:34</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D11" t="n">
         <v>77</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>46</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>109</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1143,7 +1568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1156,14 +1581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:17:32</t>
+          <t>Última actualización: 06:49:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1622,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1211,11 +1636,61 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>87</v>
+        <v>55</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>104</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>119</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1840
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:49:04</t>
+          <t>Última actualización: 07:01:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>07:01</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>62</v>
+        <v>18</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -828,16 +828,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -878,16 +878,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,12 +898,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:49:33</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>101</v>
+        <v>25</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,21 +923,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>07:34</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>40</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,21 +948,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>05:49:33</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>46</v>
+        <v>101</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>07:58</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>101</v>
+        <v>48</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1128,16 +1128,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>07:58</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:11</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>08:28</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>08:38</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1253,16 +1253,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,23 +1273,173 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>07:01:45</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>08:28</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>87</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>07:01:45</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>96</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>06:49:04</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>109</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>07:01:45</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
         <is>
           <t>08:41</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>100</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>07:01:45</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D38" t="n">
-        <v>112</v>
-      </c>
-      <c r="E38" t="inlineStr">
+      <c r="D42" t="n">
+        <v>100</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>07:01:45</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>113</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>07:01:45</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>115</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1306,7 +1456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1319,14 +1469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:49:04</t>
+          <t>Última actualización: 07:01:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1585,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1449,7 +1599,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>62</v>
+        <v>18</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1485,7 +1635,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1499,7 +1649,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1535,23 +1685,98 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>07:01:45</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>96</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>06:49:04</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>08:38</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D14" t="n">
         <v>109</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07:01:45</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>113</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>07:01:45</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>115</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1568,7 +1793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1581,14 +1806,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:49:04</t>
+          <t>Última actualización: 07:01:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1622,12 +1847,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:43</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1636,7 +1861,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1652,7 +1877,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1661,7 +1886,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1672,23 +1897,98 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>07:01:45</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:32</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>91</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>06:49:04</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>104</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:01:45</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:47</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>106</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:49:04</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>08:48</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D11" t="n">
         <v>119</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1841
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:01:45</t>
+          <t>Última actualización: 07:40:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:40</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>07:58</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>101</v>
+        <v>15</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,12 +1148,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:17:32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:58</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:17:32</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>114</v>
+        <v>19</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>76</v>
+        <v>21</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:11</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>80</v>
+        <v>31</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>08:28</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>87</v>
+        <v>41</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>08:37</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>08:38</t>
+          <t>08:28</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>109</v>
+        <v>48</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1353,16 +1353,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:37</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:38</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>08:54</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>113</v>
+        <v>61</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,23 +1423,223 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>61</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>07:40:28</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>74</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>07:40:28</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
           <t>08:56</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>76</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>07:40:28</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D44" t="n">
-        <v>115</v>
-      </c>
-      <c r="E44" t="inlineStr">
+      <c r="D47" t="n">
+        <v>76</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>07:40:28</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>87</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>07:40:28</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>97</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>07:40:28</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>97</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>07:40:28</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>106</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>07:40:28</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>09:38</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>118</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1469,7 +1669,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:01:45</t>
+          <t>Última actualización: 07:40:28</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1910,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1724,7 +1924,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1735,7 +1935,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1749,7 +1949,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1760,7 +1960,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1774,7 +1974,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>115</v>
+        <v>76</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1793,7 +1993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1806,14 +2006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:01:45</t>
+          <t>Última actualización: 07:40:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1922,7 +2122,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1936,7 +2136,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>104</v>
+        <v>53</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1972,7 +2172,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1986,11 +2186,36 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>119</v>
+        <v>68</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:40:28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>108</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1842
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:40:28</t>
+          <t>Última actualización: 08:00:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>76</v>
+        <v>21</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:11</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>08:28</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>08:37</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>08:38</t>
+          <t>08:28</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:37</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1428,16 +1428,16 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:38</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>08:54</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1478,16 +1478,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:54</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>76</v>
+        <v>54</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1528,16 +1528,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>97</v>
+        <v>56</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:02</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1603,16 +1603,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,23 +1623,248 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>08:00:48</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>71</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>08:00:48</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>77</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>07:40:28</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>97</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>08:00:48</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>77</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>08:00:48</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>86</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>08:00:48</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
         <is>
           <t>09:38</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D52" t="n">
-        <v>118</v>
-      </c>
-      <c r="E52" t="inlineStr">
+      <c r="D57" t="n">
+        <v>98</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>08:00:48</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>101</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>08:00:48</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>103</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>08:00:48</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>116</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>08:00:48</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>117</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1656,7 +1881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1669,14 +1894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:40:28</t>
+          <t>Última actualización: 08:00:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -1885,7 +2110,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1899,7 +2124,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>96</v>
+        <v>37</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1935,7 +2160,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1949,7 +2174,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1960,7 +2185,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1974,9 +2199,34 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:00:48</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>117</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1993,7 +2243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2006,14 +2256,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:40:28</t>
+          <t>Última actualización: 08:00:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2347,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2111,7 +2361,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2147,7 +2397,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2161,7 +2411,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>106</v>
+        <v>47</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2197,23 +2447,48 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>08:00:48</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>87</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>07:40:28</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>09:28</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D13" t="n">
         <v>108</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1843
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:00:48</t>
+          <t>Última actualización: 08:33:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 56</t>
+          <t>Total filas: 67</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>58</v>
+        <v>5</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>61</v>
+        <v>8</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>76</v>
+        <v>23</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>77</v>
+        <v>38</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,12 +1673,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1778,16 +1778,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:31</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>103</v>
+        <v>58</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>116</v>
+        <v>65</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,23 +1848,298 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>68</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>70</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>82</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>83</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>08:00:48</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>09:57</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D61" t="n">
+      <c r="D65" t="n">
         <v>117</v>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>85</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>87</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>98</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>100</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>113</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>114</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>10:31</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>118</v>
+      </c>
+      <c r="E72" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1881,7 +2156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1894,14 +2169,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:00:48</t>
+          <t>Última actualización: 08:33:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2410,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2149,7 +2424,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>58</v>
+        <v>5</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2160,7 +2435,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2174,7 +2449,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2185,7 +2460,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2199,7 +2474,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2227,6 +2502,31 @@
         <v>117</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>85</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2243,7 +2543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2256,14 +2556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:00:48</t>
+          <t>Última actualización: 08:33:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -2397,37 +2697,37 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>08:47</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:47</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2436,7 +2736,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2447,50 +2747,100 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>87</v>
+        <v>15</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>87</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>09:28</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>108</v>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D14" t="n">
+        <v>55</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1844
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:33:32</t>
+          <t>Última actualización: 08:50:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 67</t>
+          <t>Total filas: 73</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>08:54</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:54</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:02</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>62</v>
+        <v>6</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,12 +1598,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>09:02</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,12 +1648,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1662,7 +1662,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>38</v>
+        <v>87</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,21 +1698,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>77</v>
+        <v>21</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,12 +1748,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>86</v>
+        <v>27</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>09:31</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:31</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>82</v>
+        <v>48</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>83</v>
+        <v>51</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>117</v>
+        <v>53</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>10:13</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>09:59</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>113</v>
+        <v>69</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2103,16 +2103,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>114</v>
+        <v>87</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,23 +2123,173 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>08:50:24</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>81</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>08:50:24</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>83</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>08:50:24</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>96</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>08:50:24</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>97</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
           <t>08:33:32</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>10:31</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D72" t="n">
+      <c r="D76" t="n">
         <v>118</v>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>08:50:24</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>113</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>08:50:24</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>114</v>
+      </c>
+      <c r="E78" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2156,7 +2306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2169,14 +2319,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:33:32</t>
+          <t>Última actualización: 08:50:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2435,21 +2585,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>08:54</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2460,21 +2610,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:54</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2485,21 +2635,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>117</v>
+        <v>6</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2510,23 +2660,48 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>117</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>08:50:24</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>09:58</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>85</v>
-      </c>
-      <c r="E18" t="inlineStr">
+      <c r="D19" t="n">
+        <v>68</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2543,7 +2718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2556,14 +2731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:33:32</t>
+          <t>Última actualización: 08:50:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2772,37 +2947,37 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>08:54</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>87</v>
+        <v>4</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09:28</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2811,7 +2986,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>55</v>
+        <v>87</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2822,25 +2997,125 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>08:50:24</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>38</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>08:33:32</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>10:08</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D16" t="n">
         <v>95</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:50:24</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>83</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:50:24</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>98</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>08:50:24</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>105</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1845
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:50:24</t>
+          <t>Última actualización: 09:25:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 73</t>
+          <t>Total filas: 82</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>09:31</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:31</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1953,16 +1953,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>82</v>
+        <v>18</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>117</v>
+        <v>31</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,12 +2048,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>68</v>
+        <v>117</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>09:59</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,12 +2098,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:59</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2112,7 +2112,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10:13</t>
+          <t>10:02</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>83</v>
+        <v>37</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2178,16 +2178,16 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:11</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>10:12</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>97</v>
+        <v>47</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>10:31</t>
+          <t>10:13</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>118</v>
+        <v>48</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>113</v>
+        <v>61</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,23 +2273,248 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>62</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>08:33:32</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>10:31</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>118</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>09:25:06</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>78</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>09:25:06</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D78" t="n">
+      <c r="D81" t="n">
+        <v>79</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>09:25:06</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>85</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>09:25:06</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>91</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>09:25:06</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>93</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>09:25:06</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>105</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>09:25:06</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
         <v>114</v>
       </c>
-      <c r="E78" t="inlineStr">
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>09:25:06</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>11:22</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>117</v>
+      </c>
+      <c r="E87" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2319,7 +2544,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:50:24</t>
+          <t>Última actualización: 09:25:06</t>
         </is>
       </c>
     </row>
@@ -2685,7 +2910,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2699,7 +2924,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2718,7 +2943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2731,14 +2956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:50:24</t>
+          <t>Última actualización: 09:25:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -2972,12 +3197,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>09:25</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2986,7 +3211,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2997,12 +3222,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>09:28</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3011,7 +3236,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>38</v>
+        <v>87</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -3022,37 +3247,37 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10:08</t>
+          <t>09:28</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10:13</t>
+          <t>10:08</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3061,7 +3286,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3072,25 +3297,25 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10:28</t>
+          <t>10:12</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>98</v>
+        <v>47</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
@@ -3102,18 +3327,68 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>83</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>09:25:06</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>63</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>09:25:06</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>10:35</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>105</v>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="D21" t="n">
+        <v>70</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1846
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:25:06</t>
+          <t>Última actualización: 10:24:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 82</t>
+          <t>Total filas: 98</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2248,12 +2248,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>09:25:06</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>61</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2278,16 +2278,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>08:33:32</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>10:31</t>
+          <t>10:27</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>118</v>
+        <v>3</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>09:25:06</t>
+          <t>08:33:32</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:31</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>78</v>
+        <v>118</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>09:25:06</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>79</v>
+        <v>19</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>09:25:06</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>85</v>
+        <v>20</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2403,16 +2403,16 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>09:25:06</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>10:58</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>93</v>
+        <v>27</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2453,16 +2453,16 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>10:56</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>09:25:06</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>10:57</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>114</v>
+        <v>33</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,23 +2498,423 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>34</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>38</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>46</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>49</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
           <t>09:25:06</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>114</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>56</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>09:25:06</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
         <is>
           <t>11:22</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D87" t="n">
+      <c r="D93" t="n">
         <v>117</v>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>61</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>64</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>74</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>11:39</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>75</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>78</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>89</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>94</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>105</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>106</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>109</v>
+      </c>
+      <c r="E103" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2531,7 +2931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2544,14 +2944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:25:06</t>
+          <t>Última actualización: 10:24:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -2927,6 +3327,56 @@
         <v>33</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>64</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:39</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>75</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2943,7 +3393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2956,14 +3406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:25:06</t>
+          <t>Última actualización: 10:24:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3347,12 +3797,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>09:25:06</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10:28</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3361,7 +3811,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>63</v>
+        <v>2</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3377,20 +3827,70 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>63</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>10:35</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>70</v>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="D22" t="n">
+        <v>11</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>64</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1847
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:24:16</t>
+          <t>Última actualización: 10:57:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 98</t>
+          <t>Total filas: 110</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>11:02</t>
+          <t>10:59</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>09:25:06</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>11:13</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>114</v>
+        <v>16</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,12 +2623,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>11:19</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>56</v>
+        <v>114</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>09:25:06</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>11:22</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>117</v>
+        <v>23</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>09:25:06</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>11:25</t>
+          <t>11:22</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>61</v>
+        <v>117</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>11:28</t>
+          <t>11:25</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:27</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2753,16 +2753,16 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>11:39</t>
+          <t>11:28</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>11:42</t>
+          <t>11:38</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2803,16 +2803,16 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:38</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2828,16 +2828,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:39</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>12:09</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>105</v>
+        <v>44</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>12:10</t>
+          <t>11:42</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>106</v>
+        <v>45</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,23 +2898,323 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>56</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>58</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>61</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>71</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
           <t>10:24:16</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>105</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>106</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
         <is>
           <t>12:13</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C109" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D103" t="n">
-        <v>109</v>
-      </c>
-      <c r="E103" t="inlineStr">
+      <c r="D109" t="n">
+        <v>76</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>12:23</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>86</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>90</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>91</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>97</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>101</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>105</v>
+      </c>
+      <c r="E115" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2931,7 +3231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2944,14 +3244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:24:16</t>
+          <t>Última actualización: 10:57:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3335,12 +3635,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11:28</t>
+          <t>11:27</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3349,7 +3649,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>64</v>
+        <v>30</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3365,18 +3665,93 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>64</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>41</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10:24:16</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>11:39</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D23" t="n">
         <v>75</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>90</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3393,7 +3768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3406,14 +3781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:24:16</t>
+          <t>Última actualización: 10:57:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3872,23 +4247,48 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>30</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>10:24:16</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>11:28</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D24" t="n">
         <v>64</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1848
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E115"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:57:43</t>
+          <t>Última actualización: 11:23:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 110</t>
+          <t>Total filas: 116</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>41</v>
+        <v>74</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2862,7 +2862,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2912,7 +2912,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2962,7 +2962,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>71</v>
+        <v>45</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,12 +3123,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -3137,7 +3137,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>91</v>
+        <v>61</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>97</v>
+        <v>64</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3178,16 +3178,16 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,23 +3198,173 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
+          <t>11:23:38</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>70</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
           <t>10:57:43</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>97</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>11:23:38</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>75</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>11:23:38</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
         <is>
           <t>12:42</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
+      <c r="C118" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D115" t="n">
-        <v>105</v>
-      </c>
-      <c r="E115" t="inlineStr">
+      <c r="D118" t="n">
+        <v>79</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>11:23:38</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>93</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>11:23:38</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>110</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>11:23:38</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>111</v>
+      </c>
+      <c r="E121" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3244,7 +3394,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:57:43</t>
+          <t>Última actualización: 11:23:38</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3785,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3649,7 +3799,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3685,7 +3835,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3699,7 +3849,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3735,7 +3885,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3749,7 +3899,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -3768,7 +3918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3781,14 +3931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:57:43</t>
+          <t>Última actualización: 11:23:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4247,12 +4397,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>11:27</t>
+          <t>11:24</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4261,7 +4411,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4272,23 +4422,73 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>10:57:43</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>30</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>10:24:16</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>11:28</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D25" t="n">
         <v>64</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>11:23:38</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>94</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1849
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:23:38</t>
+          <t>Última actualización: 11:50:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 116</t>
+          <t>Total filas: 126</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2898,12 +2898,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:50</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2912,7 +2912,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2928,16 +2928,16 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,12 +2998,12 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>12:09</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>105</v>
+        <v>18</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3028,16 +3028,16 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>12:10</t>
+          <t>12:09</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>12:13</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,12 +3073,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:13</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3103,16 +3103,16 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:18</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>61</v>
+        <v>28</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,12 +3173,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -3187,7 +3187,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>91</v>
+        <v>61</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>70</v>
+        <v>37</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3228,16 +3228,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>75</v>
+        <v>41</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3278,16 +3278,16 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>110</v>
+        <v>46</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,23 +3348,273 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>48</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>52</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>66</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>67</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>83</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
           <t>13:14</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr">
+      <c r="C126" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D121" t="n">
-        <v>111</v>
-      </c>
-      <c r="E121" t="inlineStr">
+      <c r="D126" t="n">
+        <v>84</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>93</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>94</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>102</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>110</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>117</v>
+      </c>
+      <c r="E131" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3381,7 +3631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3394,14 +3644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:23:38</t>
+          <t>Última actualización: 11:50:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -3885,7 +4135,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3899,9 +4149,59 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>64</v>
+        <v>37</v>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>67</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>94</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3918,7 +4218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3931,14 +4231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:23:38</t>
+          <t>Última actualización: 11:50:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4772,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4486,11 +4786,36 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>11:50:46</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>98</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1850
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E131"/>
+  <dimension ref="A1:E136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:50:46</t>
+          <t>Última actualización: 12:15:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 126</t>
+          <t>Total filas: 131</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,12 +3123,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>12:18</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -3137,7 +3137,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3153,16 +3153,16 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:18</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,12 +3223,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>91</v>
+        <v>61</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>10:57:43</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>97</v>
+        <v>16</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,12 +3323,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>10:57:43</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>48</v>
+        <v>97</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:38</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:42</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>67</v>
+        <v>27</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>84</v>
+        <v>41</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>93</v>
+        <v>42</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>94</v>
+        <v>58</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>102</v>
+        <v>59</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3578,16 +3578,16 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,23 +3598,148 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>69</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>12:15:43</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>70</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>12:15:43</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>77</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>12:15:43</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>85</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>12:15:43</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
           <t>13:47</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr">
+      <c r="C135" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D131" t="n">
-        <v>117</v>
-      </c>
-      <c r="E131" t="inlineStr">
+      <c r="D135" t="n">
+        <v>92</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>12:15:43</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>95</v>
+      </c>
+      <c r="E136" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3644,7 +3769,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:50:46</t>
+          <t>Última actualización: 12:15:43</t>
         </is>
       </c>
     </row>
@@ -4135,7 +4260,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4149,7 +4274,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4160,7 +4285,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4174,7 +4299,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4185,7 +4310,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4199,7 +4324,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4218,7 +4343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4231,14 +4356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:50:46</t>
+          <t>Última actualización: 12:15:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4772,7 +4897,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4786,7 +4911,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4797,7 +4922,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4811,11 +4936,36 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>12:15:43</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>97</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1851
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E136"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:15:43</t>
+          <t>Última actualización: 12:42:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 131</t>
+          <t>Total filas: 141</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:42:31</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,12 +3448,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:42:31</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:42</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3462,7 +3462,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:42:31</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>41</v>
+        <v>13</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:42:31</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3528,16 +3528,16 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:42:31</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:42:31</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>93</v>
+        <v>31</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:42:31</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>69</v>
+        <v>32</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,12 +3623,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:42:31</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:42:31</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>85</v>
+        <v>42</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3703,16 +3703,16 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,23 +3723,273 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:42:31</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>50</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>58</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>65</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
           <t>13:50</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr">
+      <c r="C139" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D136" t="n">
-        <v>95</v>
-      </c>
-      <c r="E136" t="inlineStr">
+      <c r="D139" t="n">
+        <v>68</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>86</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>86</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>89</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>94</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>104</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>106</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>119</v>
+      </c>
+      <c r="E146" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3756,7 +4006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3769,14 +4019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:15:43</t>
+          <t>Última actualización: 12:42:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4310,23 +4560,73 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:42:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>16</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>13:24</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>69</v>
-      </c>
-      <c r="E26" t="inlineStr">
+      <c r="D27" t="n">
+        <v>42</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>106</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4343,7 +4643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4356,14 +4656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:15:43</t>
+          <t>Última actualización: 12:42:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -4897,12 +5197,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:42:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -4911,7 +5211,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4927,20 +5227,20 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>73</v>
+        <v>42</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
@@ -4952,18 +5252,93 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>73</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>13:29</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>47</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>12:15:43</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>13:52</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D30" t="n">
         <v>97</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>12:42:31</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>71</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1852
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E146"/>
+  <dimension ref="A1:E151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:42:31</t>
+          <t>Última actualización: 12:58:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 141</t>
+          <t>Total filas: 146</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:59</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,12 +3648,12 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:50:46</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3662,7 +3662,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>93</v>
+        <v>23</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>11:50:46</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>42</v>
+        <v>93</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:40</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>104</v>
+        <v>73</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>106</v>
+        <v>78</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,23 +3973,148 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>88</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>12:58:35</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>90</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>12:58:35</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
           <t>14:41</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr">
+      <c r="C148" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D146" t="n">
-        <v>119</v>
-      </c>
-      <c r="E146" t="inlineStr">
+      <c r="D148" t="n">
+        <v>103</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>12:58:35</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>110</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>12:58:35</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>117</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>12:58:35</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>118</v>
+      </c>
+      <c r="E151" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4006,7 +4131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4019,14 +4144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:42:31</t>
+          <t>Última actualización: 12:58:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -4585,21 +4710,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>12:59</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4610,23 +4735,98 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>26</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>12:58:35</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>14:28</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>106</v>
-      </c>
-      <c r="E28" t="inlineStr">
+      <c r="D29" t="n">
+        <v>90</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>12:58:35</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>110</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>12:58:35</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>118</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4643,7 +4843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4656,14 +4856,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:42:31</t>
+          <t>Última actualización: 12:58:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -5247,37 +5447,37 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>73</v>
+        <v>2</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12:42:31</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>13:29</t>
+          <t>13:28</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -5286,7 +5486,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5297,48 +5497,73 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>12:58:35</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>13:52</t>
+          <t>13:29</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>97</v>
+        <v>31</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>12:58:35</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>54</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>12:42:31</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>13:53</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D32" t="n">
         <v>71</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1853
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E151"/>
+  <dimension ref="A1:E159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:58:35</t>
+          <t>Última actualización: 13:27:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 146</t>
+          <t>Total filas: 154</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3762,7 +3762,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3812,7 +3812,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,7 +3823,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3837,7 +3837,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,7 +3848,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>73</v>
+        <v>44</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3962,7 +3962,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>78</v>
+        <v>49</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>90</v>
+        <v>59</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>103</v>
+        <v>60</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4053,16 +4053,16 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>117</v>
+        <v>74</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,23 +4098,223 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>80</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
           <t>12:58:35</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>110</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>12:58:35</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>117</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
         <is>
           <t>14:56</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
+      <c r="C154" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D151" t="n">
-        <v>118</v>
-      </c>
-      <c r="E151" t="inlineStr">
+      <c r="D154" t="n">
+        <v>89</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>92</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>100</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>103</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>104</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>119</v>
+      </c>
+      <c r="E159" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4131,7 +4331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4144,14 +4344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:58:35</t>
+          <t>Última actualización: 13:27:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -4760,12 +4960,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -4774,7 +4974,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -4790,16 +4990,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -4810,23 +5010,73 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>80</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>12:58:35</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>110</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>14:56</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>118</v>
-      </c>
-      <c r="E31" t="inlineStr">
+      <c r="D33" t="n">
+        <v>89</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4843,7 +5093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4856,14 +5106,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:58:35</t>
+          <t>Última actualización: 13:27:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5472,7 +5722,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5486,7 +5736,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5522,7 +5772,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5536,7 +5786,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -5566,6 +5816,56 @@
       <c r="E32" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>60</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>15:12</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>105</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1854
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E159"/>
+  <dimension ref="A1:E169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:27:47</t>
+          <t>Última actualización: 13:54:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 154</t>
+          <t>Total filas: 164</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3848,12 +3848,12 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:54</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3878,16 +3878,16 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3953,16 +3953,16 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4003,16 +4003,16 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4078,16 +4078,16 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>117</v>
+        <v>34</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4203,16 +4203,16 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>100</v>
+        <v>54</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4278,16 +4278,16 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,23 +4298,273 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>63</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
           <t>13:27:47</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr">
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>92</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>15:02</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>68</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>73</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>76</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>77</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
         <is>
           <t>15:26</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
+      <c r="C165" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D159" t="n">
+      <c r="D165" t="n">
         <v>119</v>
       </c>
-      <c r="E159" t="inlineStr">
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>93</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>94</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>15:39</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>105</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>114</v>
+      </c>
+      <c r="E169" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4331,7 +4581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4344,14 +4594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:27:47</t>
+          <t>Última actualización: 13:54:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -4985,7 +5235,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4999,7 +5249,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5035,7 +5285,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>12:58:35</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5049,7 +5299,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>110</v>
+        <v>54</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5077,6 +5327,56 @@
         <v>89</v>
       </c>
       <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>63</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>94</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5093,7 +5393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5106,14 +5406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:27:47</t>
+          <t>Última actualización: 13:54:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -5822,12 +6122,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>13:54</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5836,7 +6136,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5852,18 +6152,93 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>60</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>34</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>13:27:47</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>15:12</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D36" t="n">
         <v>105</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>79</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1855
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E169"/>
+  <dimension ref="A1:E177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:54:07</t>
+          <t>Última actualización: 14:16:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 164</t>
+          <t>Total filas: 172</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4008,11 +4008,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,12 +4023,12 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>59</v>
+        <v>9</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,12 +4098,12 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -4112,7 +4112,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4153,16 +4153,16 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4178,16 +4178,16 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,12 +4223,12 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>54</v>
+        <v>80</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,12 +4298,12 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -4312,7 +4312,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:57</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>92</v>
+        <v>63</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,12 +4348,12 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>15:02</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -4362,7 +4362,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4403,16 +4403,16 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>119</v>
+        <v>54</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>93</v>
+        <v>55</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15:39</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4553,18 +4553,218 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>93</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>94</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>14:16:36</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>82</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>13:54:07</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>15:39</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>105</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>14:16:36</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
           <t>15:48</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr">
+      <c r="C173" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D169" t="n">
-        <v>114</v>
-      </c>
-      <c r="E169" t="inlineStr">
+      <c r="D173" t="n">
+        <v>92</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>14:16:36</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>100</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>14:16:36</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>100</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>14:16:36</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>111</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>14:16:36</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>118</v>
+      </c>
+      <c r="E177" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4581,7 +4781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4594,14 +4794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:54:07</t>
+          <t>Última actualización: 14:16:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -5210,7 +5410,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5224,7 +5424,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5285,7 +5485,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5299,7 +5499,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5310,7 +5510,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5324,7 +5524,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>89</v>
+        <v>40</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5360,23 +5560,48 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>14:16:36</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>71</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>13:54:07</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>15:28</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D36" t="n">
         <v>94</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5393,7 +5618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5406,14 +5631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:54:07</t>
+          <t>Última actualización: 14:16:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -6147,7 +6372,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6161,7 +6386,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6222,7 +6447,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6236,11 +6461,36 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>14:16:36</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>15:52</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>96</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1856
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E177"/>
+  <dimension ref="A1:E189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:16:36</t>
+          <t>Última actualización: 14:44:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 172</t>
+          <t>Total filas: 184</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,12 +4248,12 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,12 +4323,12 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>13:27:47</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:57</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>92</v>
+        <v>13</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,12 +4373,12 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:27:47</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -4387,7 +4387,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>45</v>
+        <v>92</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,12 +4398,12 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>15:02</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>71</v>
+        <v>41</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,12 +4548,12 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -4562,7 +4562,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,12 +4573,12 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>94</v>
+        <v>71</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>82</v>
+        <v>43</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>15:39</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>105</v>
+        <v>44</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4653,16 +4653,16 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:39</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>100</v>
+        <v>57</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>111</v>
+        <v>64</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,23 +4748,323 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
+          <t>14:44:16</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>15:52</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>68</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
           <t>14:16:36</t>
         </is>
       </c>
-      <c r="B177" t="inlineStr">
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>100</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>14:16:36</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>100</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>14:44:16</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>73</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>14:44:16</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>81</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>14:44:16</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>83</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>14:44:16</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>16:09</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>85</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>14:16:36</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
         <is>
           <t>16:14</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
+      <c r="C184" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D177" t="n">
+      <c r="D184" t="n">
         <v>118</v>
       </c>
-      <c r="E177" t="inlineStr">
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>14:44:16</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>99</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>14:44:16</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>16:27</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>103</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>14:44:16</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>114</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>14:44:16</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>116</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>14:44:16</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>117</v>
+      </c>
+      <c r="E189" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4794,7 +5094,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:16:36</t>
+          <t>Última actualización: 14:44:16</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5785,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5499,7 +5799,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5535,7 +5835,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5549,7 +5849,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -5585,7 +5885,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5599,7 +5899,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>94</v>
+        <v>44</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -5618,7 +5918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5631,14 +5931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:16:36</t>
+          <t>Última actualización: 14:44:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6747,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6461,7 +6761,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6491,6 +6791,56 @@
       <c r="E38" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>14:44:16</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>69</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>14:44:16</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>114</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1857
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E189"/>
+  <dimension ref="A1:E195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:44:16</t>
+          <t>Última actualización: 14:59:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 184</t>
+          <t>Total filas: 190</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4448,7 +4448,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>73</v>
+        <v>100</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>83</v>
+        <v>58</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>118</v>
+        <v>81</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>99</v>
+        <v>68</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4978,16 +4978,16 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>16:27</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>114</v>
+        <v>72</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,23 +5048,173 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>84</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>14:59:09</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>16:27</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>88</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>14:59:09</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>99</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>14:59:09</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>101</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>14:59:09</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
           <t>16:41</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr">
+      <c r="C193" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D189" t="n">
-        <v>117</v>
-      </c>
-      <c r="E189" t="inlineStr">
+      <c r="D193" t="n">
+        <v>102</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>14:59:09</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>114</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>14:59:09</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>16:57</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>118</v>
+      </c>
+      <c r="E195" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5094,7 +5244,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:44:16</t>
+          <t>Última actualización: 14:59:09</t>
         </is>
       </c>
     </row>
@@ -5885,7 +6035,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5899,7 +6049,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -5931,7 +6081,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:44:16</t>
+          <t>Última actualización: 14:59:09</t>
         </is>
       </c>
     </row>
@@ -6747,7 +6897,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6761,7 +6911,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6797,7 +6947,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6811,7 +6961,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6822,7 +6972,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6836,7 +6986,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1858
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E195"/>
+  <dimension ref="A1:E203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:59:09</t>
+          <t>Última actualización: 15:36:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 190</t>
+          <t>Total filas: 198</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4583,11 +4583,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>42</v>
+        <v>5</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,12 +4848,12 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>58</v>
+        <v>100</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,7 +4873,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -4883,11 +4883,11 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4903,16 +4903,16 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,12 +4923,12 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4937,7 +4937,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>14:44:16</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>85</v>
+        <v>31</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,12 +4998,12 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>14:44:16</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,12 +5023,12 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>118</v>
+        <v>35</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>84</v>
+        <v>118</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>16:27</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>88</v>
+        <v>47</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>99</v>
+        <v>49</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:26</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>101</v>
+        <v>50</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5153,16 +5153,16 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:27</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:38</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>114</v>
+        <v>62</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,23 +5198,223 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
+          <t>15:36:22</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>64</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>15:36:22</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>65</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>15:36:22</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>65</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>15:36:22</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>77</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>15:36:22</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>80</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
           <t>14:59:09</t>
         </is>
       </c>
-      <c r="B195" t="inlineStr">
+      <c r="B200" t="inlineStr">
         <is>
           <t>16:57</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr">
+      <c r="C200" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D195" t="n">
+      <c r="D200" t="n">
         <v>118</v>
       </c>
-      <c r="E195" t="inlineStr">
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>15:36:22</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>92</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>15:36:22</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>106</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>15:36:22</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>116</v>
+      </c>
+      <c r="E203" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5231,7 +5431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5244,14 +5444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:59:09</t>
+          <t>Última actualización: 15:36:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -6052,6 +6252,56 @@
         <v>29</v>
       </c>
       <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>15:36:22</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>92</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>15:36:22</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>116</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6068,7 +6318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6081,14 +6331,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:59:09</t>
+          <t>Última actualización: 15:36:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -6947,7 +7197,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6961,7 +7211,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6972,7 +7222,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6986,11 +7236,36 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>99</v>
+        <v>62</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>15:36:22</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>17:03</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>87</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1859
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E203"/>
+  <dimension ref="A1:E210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:36:22</t>
+          <t>Última actualización: 16:03:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 198</t>
+          <t>Total filas: 205</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4583,11 +4583,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5112,7 +5112,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>62</v>
+        <v>35</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>64</v>
+        <v>37</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5287,7 +5287,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>80</v>
+        <v>52</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,12 +5323,12 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>16:57</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -5337,7 +5337,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>118</v>
+        <v>53</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>92</v>
+        <v>118</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5403,18 +5403,193 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>92</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>16:03:48</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>79</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>16:03:48</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
           <t>17:32</t>
         </is>
       </c>
-      <c r="C203" t="inlineStr">
+      <c r="C205" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D203" t="n">
-        <v>116</v>
-      </c>
-      <c r="E203" t="inlineStr">
+      <c r="D205" t="n">
+        <v>89</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>16:03:48</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>93</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>16:03:48</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>95</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>16:03:48</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>17:39</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>96</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>16:03:48</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>107</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>16:03:48</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>17:52</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>109</v>
+      </c>
+      <c r="E210" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5431,7 +5606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5444,14 +5619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:36:22</t>
+          <t>Última actualización: 16:03:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -6260,12 +6435,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -6274,7 +6449,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6290,18 +6465,68 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>92</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>16:03:48</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>17:32</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D38" t="n">
-        <v>116</v>
-      </c>
-      <c r="E38" t="inlineStr">
+      <c r="D39" t="n">
+        <v>89</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>16:03:48</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>17:52</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>109</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6318,7 +6543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6331,14 +6556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:36:22</t>
+          <t>Última actualización: 16:03:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -7222,12 +7447,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:37</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -7236,7 +7461,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7252,18 +7477,68 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>62</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>16:03:48</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>17:02</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>59</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>15:36:22</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>17:03</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D41" t="n">
+      <c r="D43" t="n">
         <v>87</v>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1860
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E210"/>
+  <dimension ref="A1:E220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:03:48</t>
+          <t>Última actualización: 16:35:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 205</t>
+          <t>Total filas: 215</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -4873,7 +4873,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -4883,11 +4883,11 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -5173,12 +5173,12 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5203,16 +5203,16 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:38</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:43</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:53</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>16:57</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>118</v>
+        <v>20</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>92</v>
+        <v>118</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>89</v>
+        <v>33</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>93</v>
+        <v>47</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>95</v>
+        <v>50</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>17:39</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>96</v>
+        <v>57</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>107</v>
+        <v>61</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,23 +5573,273 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>63</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
           <t>16:03:48</t>
         </is>
       </c>
-      <c r="B210" t="inlineStr">
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>17:39</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>96</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>72</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>75</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>16:03:48</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
         <is>
           <t>17:52</t>
         </is>
       </c>
-      <c r="C210" t="inlineStr">
+      <c r="C214" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D210" t="n">
+      <c r="D214" t="n">
         <v>109</v>
       </c>
-      <c r="E210" t="inlineStr">
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>78</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>90</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>93</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>95</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>105</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>108</v>
+      </c>
+      <c r="E220" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5606,7 +5856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5619,14 +5869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:03:48</t>
+          <t>Última actualización: 16:35:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -6460,7 +6710,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6474,7 +6724,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>92</v>
+        <v>33</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6485,7 +6735,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6499,7 +6749,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>89</v>
+        <v>57</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6527,6 +6777,56 @@
         <v>109</v>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>78</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>108</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6543,7 +6843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6556,14 +6856,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:03:48</t>
+          <t>Última actualización: 16:35:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -7447,12 +7747,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>16:37</t>
+          <t>16:36</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -7461,7 +7761,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7472,12 +7772,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:37</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -7486,7 +7786,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7497,48 +7797,98 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>17:02</t>
+          <t>16:38</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>17:02</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>27</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>15:36:22</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>17:03</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D43" t="n">
+      <c r="D44" t="n">
         <v>87</v>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>16:35:34</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>18:29</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>114</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1861
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E220"/>
+  <dimension ref="A1:E226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:35:34</t>
+          <t>Última actualización: 16:50:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 215</t>
+          <t>Total filas: 221</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4583,11 +4583,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5337,7 +5337,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>118</v>
+        <v>7</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5462,7 +5462,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5578,16 +5578,16 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>17:39</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>96</v>
+        <v>47</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>109</v>
+        <v>57</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>93</v>
+        <v>63</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5778,16 +5778,16 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,23 +5823,173 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>78</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>16:50:15</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>80</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>16:50:15</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>90</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>16:50:15</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
           <t>18:23</t>
         </is>
       </c>
-      <c r="C220" t="inlineStr">
+      <c r="C223" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D220" t="n">
-        <v>108</v>
-      </c>
-      <c r="E220" t="inlineStr">
+      <c r="D223" t="n">
+        <v>93</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>16:50:15</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>18:27</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>97</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>16:50:15</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>106</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>16:50:15</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>107</v>
+      </c>
+      <c r="E226" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5856,7 +6006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5869,14 +6019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:35:34</t>
+          <t>Última actualización: 16:50:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -6710,7 +6860,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6724,7 +6874,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6760,21 +6910,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>109</v>
+        <v>43</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -6785,12 +6935,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -6799,7 +6949,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -6810,23 +6960,48 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>63</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>16:50:15</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>18:23</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D42" t="n">
-        <v>108</v>
-      </c>
-      <c r="E42" t="inlineStr">
+      <c r="D43" t="n">
+        <v>93</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6843,7 +7018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6856,14 +7031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:35:34</t>
+          <t>Última actualización: 16:50:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -7847,7 +8022,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7861,7 +8036,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>87</v>
+        <v>13</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7889,6 +8064,31 @@
         <v>114</v>
       </c>
       <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>16:50:15</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>100</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1862
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E226"/>
+  <dimension ref="A1:E235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:50:15</t>
+          <t>Última actualización: 16:58:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 221</t>
+          <t>Total filas: 230</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -5423,7 +5423,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>64</v>
+        <v>9</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,12 +5548,12 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -5562,7 +5562,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,12 +5598,12 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -5612,7 +5612,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5628,16 +5628,16 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>17:39</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>96</v>
+        <v>39</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5678,16 +5678,16 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>60</v>
+        <v>96</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>109</v>
+        <v>57</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:49</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>18:06</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>76</v>
+        <v>54</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5828,16 +5828,16 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5878,16 +5878,16 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:07</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5928,16 +5928,16 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>18:27</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,23 +5973,248 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>18:19</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>81</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
           <t>16:50:15</t>
         </is>
       </c>
-      <c r="B226" t="inlineStr">
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>90</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>84</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>16:50:15</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>93</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>87</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>18:27</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>89</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>97</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>16:50:15</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>106</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
         <is>
           <t>18:37</t>
         </is>
       </c>
-      <c r="C226" t="inlineStr">
+      <c r="C234" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D226" t="n">
-        <v>107</v>
-      </c>
-      <c r="E226" t="inlineStr">
+      <c r="D234" t="n">
+        <v>99</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>18:52</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>114</v>
+      </c>
+      <c r="E235" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6006,7 +6231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6019,14 +6244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:50:15</t>
+          <t>Última actualización: 16:58:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -6835,7 +7060,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6849,7 +7074,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>64</v>
+        <v>9</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6885,7 +7110,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6899,7 +7124,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6935,7 +7160,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -6949,7 +7174,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>109</v>
+        <v>54</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -6985,23 +7210,48 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>16:58:56</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>84</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>16:50:15</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>18:23</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D43" t="n">
+      <c r="D44" t="n">
         <v>93</v>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7031,7 +7281,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:50:15</t>
+          <t>Última actualización: 16:58:56</t>
         </is>
       </c>
     </row>
@@ -7997,7 +8247,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8011,7 +8261,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8047,7 +8297,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8061,7 +8311,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1863
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E235"/>
+  <dimension ref="A1:E244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:58:56</t>
+          <t>Última actualización: 17:26:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 230</t>
+          <t>Total filas: 239</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4583,11 +4583,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -4873,7 +4873,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -4883,11 +4883,11 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5553,16 +5553,16 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,12 +5573,12 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,12 +5623,12 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -5637,7 +5637,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5678,16 +5678,16 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>17:39</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>96</v>
+        <v>39</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>17:49</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5778,16 +5778,16 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5803,16 +5803,16 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:49</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5853,16 +5853,16 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>18:06</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>76</v>
+        <v>27</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>18:07</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>69</v>
+        <v>39</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5928,16 +5928,16 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5953,16 +5953,16 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>18:07</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>18:19</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>90</v>
+        <v>44</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6028,16 +6028,16 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:19</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>93</v>
+        <v>54</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6078,16 +6078,16 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>18:27</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>89</v>
+        <v>57</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6128,16 +6128,16 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:27</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:28</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>99</v>
+        <v>62</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,23 +6198,248 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>69</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>16:50:15</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>106</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>71</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
           <t>16:58:56</t>
         </is>
       </c>
-      <c r="B235" t="inlineStr">
+      <c r="B238" t="inlineStr">
         <is>
           <t>18:52</t>
         </is>
       </c>
-      <c r="C235" t="inlineStr">
+      <c r="C238" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D235" t="n">
+      <c r="D238" t="n">
         <v>114</v>
       </c>
-      <c r="E235" t="inlineStr">
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>87</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>99</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>102</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>110</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>115</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>117</v>
+      </c>
+      <c r="E244" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6231,7 +6456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6244,14 +6469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:58:56</t>
+          <t>Última actualización: 17:26:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -7110,7 +7335,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7124,7 +7349,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -7185,7 +7410,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7199,7 +7424,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7235,7 +7460,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7249,9 +7474,59 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>102</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>117</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7268,7 +7543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7281,14 +7556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:58:56</t>
+          <t>Última actualización: 17:26:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8597,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8336,11 +8611,36 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>100</v>
+        <v>64</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>19:02</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>96</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1864
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E244"/>
+  <dimension ref="A1:E255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:26:32</t>
+          <t>Última actualización: 17:49:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 239</t>
+          <t>Total filas: 250</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5848,7 +5848,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>54</v>
+        <v>3</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6012,7 +6012,7 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6048,7 +6048,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -6062,7 +6062,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>84</v>
+        <v>32</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,12 +6098,12 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -6112,7 +6112,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>18:27</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6178,16 +6178,16 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>18:28</t>
+          <t>18:27</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6203,16 +6203,16 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:28</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,12 +6223,12 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -6237,7 +6237,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>106</v>
+        <v>46</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>18:52</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>114</v>
+        <v>48</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:52</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>102</v>
+        <v>64</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>110</v>
+        <v>66</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>115</v>
+        <v>75</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6428,18 +6428,293 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>99</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>17:49:49</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>78</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>102</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>17:49:49</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>19:11</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>82</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>110</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>17:49:49</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>19:20</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>91</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>17:49:49</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>92</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>17:49:49</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>93</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
           <t>19:23</t>
         </is>
       </c>
-      <c r="C244" t="inlineStr">
+      <c r="C252" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D244" t="n">
+      <c r="D252" t="n">
         <v>117</v>
       </c>
-      <c r="E244" t="inlineStr">
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>17:49:49</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>111</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>17:49:49</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>112</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>17:49:49</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>114</v>
+      </c>
+      <c r="E255" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6456,7 +6731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6469,14 +6744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:26:32</t>
+          <t>Última actualización: 17:49:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -7385,7 +7660,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7399,7 +7674,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>54</v>
+        <v>3</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7435,7 +7710,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7449,7 +7724,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>84</v>
+        <v>33</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -7485,12 +7760,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -7499,7 +7774,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -7515,18 +7790,68 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>102</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>17:49:49</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>93</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>17:26:32</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>19:23</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D46" t="n">
+      <c r="D48" t="n">
         <v>117</v>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7543,7 +7868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7556,14 +7881,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:26:32</t>
+          <t>Última actualización: 17:49:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -8572,7 +8897,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8586,7 +8911,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>91</v>
+        <v>40</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -8622,23 +8947,48 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>17:49:49</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>19:01</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>72</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>17:26:32</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>19:02</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D47" t="n">
+      <c r="D48" t="n">
         <v>96</v>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1865
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E255"/>
+  <dimension ref="A1:E259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:49:49</t>
+          <t>Última actualización: 18:03:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 250</t>
+          <t>Total filas: 254</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4583,11 +4583,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -4873,7 +4873,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -4883,11 +4883,11 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>18:03</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,12 +5923,12 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>18:06</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>76</v>
+        <v>2</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>18:07</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,12 +5973,12 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>18:07</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>18:19</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>81</v>
+        <v>7</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,12 +6048,12 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:19</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -6062,7 +6062,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>31</v>
+        <v>81</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6103,16 +6103,16 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,12 +6123,12 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -6137,7 +6137,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,12 +6173,12 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>18:27</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -6187,7 +6187,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,12 +6198,12 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>18:28</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -6212,7 +6212,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:27</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:28</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>61</v>
+        <v>106</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>18:52</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>114</v>
+        <v>34</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:52</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>66</v>
+        <v>114</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,21 +6423,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6453,16 +6453,16 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>19:07</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>102</v>
+        <v>62</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6528,16 +6528,16 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6553,16 +6553,16 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,21 +6598,21 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>112</v>
+        <v>79</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,23 +6698,123 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>117</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>18:03:44</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>97</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>18:03:44</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>98</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>18:03:44</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
           <t>19:43</t>
         </is>
       </c>
-      <c r="C255" t="inlineStr">
+      <c r="C258" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D255" t="n">
-        <v>114</v>
-      </c>
-      <c r="E255" t="inlineStr">
+      <c r="D258" t="n">
+        <v>100</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>18:03:44</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>118</v>
+      </c>
+      <c r="E259" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6731,7 +6831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6744,14 +6844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:49:49</t>
+          <t>Última actualización: 18:03:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -7710,21 +7810,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:03</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -7735,12 +7835,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -7749,7 +7849,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7760,21 +7860,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>19:07</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -7785,12 +7885,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -7799,7 +7899,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>102</v>
+        <v>64</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -7810,21 +7910,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -7835,23 +7935,48 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>18:03:44</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>79</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>17:26:32</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>19:23</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D48" t="n">
+      <c r="D49" t="n">
         <v>117</v>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7868,7 +7993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7881,14 +8006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:49:49</t>
+          <t>Última actualización: 18:03:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -8897,7 +9022,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8911,7 +9036,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -8947,7 +9072,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8961,7 +9086,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -8991,6 +9116,31 @@
       <c r="E48" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>18:03:44</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>118</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1866
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E259"/>
+  <dimension ref="A1:E267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:03:44</t>
+          <t>Última actualización: 18:35:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 254</t>
+          <t>Total filas: 262</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4583,11 +4583,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -6273,7 +6273,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6323,7 +6323,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -6337,7 +6337,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,12 +6348,12 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:49</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -6362,7 +6362,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>18:52</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>114</v>
+        <v>47</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,12 +6398,12 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:52</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -6412,7 +6412,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,21 +6423,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,12 +6473,12 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -6487,7 +6487,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6503,16 +6503,16 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>19:07</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,12 +6523,12 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -6537,7 +6537,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>102</v>
+        <v>32</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>110</v>
+        <v>36</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,12 +6598,12 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -6612,7 +6612,7 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>75</v>
+        <v>41</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,12 +6623,12 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -6637,7 +6637,7 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,12 +6698,12 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -6712,7 +6712,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>117</v>
+        <v>47</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,21 +6723,21 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>97</v>
+        <v>117</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,21 +6748,21 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>98</v>
+        <v>55</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,23 +6798,223 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
+          <t>18:35:56</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>65</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
           <t>18:03:44</t>
         </is>
       </c>
-      <c r="B259" t="inlineStr">
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>98</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>18:35:56</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>68</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>18:35:56</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>19:58</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>83</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>18:35:56</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
         <is>
           <t>20:01</t>
         </is>
       </c>
-      <c r="C259" t="inlineStr">
+      <c r="C263" t="inlineStr">
         <is>
           <t>23_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D259" t="n">
-        <v>118</v>
-      </c>
-      <c r="E259" t="inlineStr">
+      <c r="D263" t="n">
+        <v>86</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>18:35:56</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>87</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>18:35:56</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>87</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>18:35:56</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>107</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>18:35:56</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>20:24</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>109</v>
+      </c>
+      <c r="E267" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6831,7 +7031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6844,14 +7044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:03:44</t>
+          <t>Última actualización: 18:35:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -7885,7 +8085,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7899,7 +8099,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -7935,7 +8135,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7949,7 +8149,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>79</v>
+        <v>47</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -7977,6 +8177,31 @@
         <v>117</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>18:35:56</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>87</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8006,7 +8231,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:03:44</t>
+          <t>Última actualización: 18:35:56</t>
         </is>
       </c>
     </row>
@@ -9072,7 +9297,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -9086,7 +9311,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -9122,7 +9347,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -9136,7 +9361,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1867
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E267"/>
+  <dimension ref="A1:E273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:35:56</t>
+          <t>Última actualización: 18:53:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 262</t>
+          <t>Total filas: 268</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4873,7 +4873,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -4883,11 +4883,11 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6498,7 +6498,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -6512,7 +6512,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -6537,7 +6537,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6598,7 +6598,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -6612,7 +6612,7 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,12 +6723,12 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -6737,7 +6737,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>117</v>
+        <v>29</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,21 +6748,21 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>55</v>
+        <v>117</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6803,16 +6803,16 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,12 +6823,12 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -6837,7 +6837,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>98</v>
+        <v>65</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,21 +6873,21 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>19:58</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6928,16 +6928,16 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:58</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>107</v>
+        <v>68</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,23 +6998,173 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
+          <t>18:53:42</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>69</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>18:53:42</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>69</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>18:53:42</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>89</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
           <t>18:35:56</t>
         </is>
       </c>
-      <c r="B267" t="inlineStr">
+      <c r="B270" t="inlineStr">
         <is>
           <t>20:24</t>
         </is>
       </c>
-      <c r="C267" t="inlineStr">
+      <c r="C270" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D267" t="n">
+      <c r="D270" t="n">
         <v>109</v>
       </c>
-      <c r="E267" t="inlineStr">
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>18:53:42</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>92</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>18:53:42</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>20:43</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>110</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>18:53:42</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>112</v>
+      </c>
+      <c r="E273" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7031,7 +7181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7044,14 +7194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:35:56</t>
+          <t>Última actualización: 18:53:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -8085,7 +8235,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8099,7 +8249,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8135,7 +8285,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8149,7 +8299,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -8185,7 +8335,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -8199,9 +8349,34 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>18:53:42</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>20:43</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>110</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8218,7 +8393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8231,14 +8406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:35:56</t>
+          <t>Última actualización: 18:53:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -9297,7 +9472,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -9311,7 +9486,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -9347,7 +9522,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -9361,9 +9536,34 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>18:53:42</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>108</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1868
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E273"/>
+  <dimension ref="A1:E282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:42</t>
+          <t>Última actualización: 19:14:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 268</t>
+          <t>Total filas: 277</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4858,7 +4858,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,7 +6173,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -6183,11 +6183,11 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6623,12 +6623,12 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -6637,7 +6637,7 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>75</v>
+        <v>3</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6673,12 +6673,12 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>17:49:49</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -6687,7 +6687,7 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>17:49:49</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,21 +6723,21 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,12 +6748,12 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -6762,7 +6762,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>117</v>
+        <v>29</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,12 +6798,12 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -6812,7 +6812,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6828,16 +6828,16 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,7 +6848,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -6862,7 +6862,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,12 +6873,12 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>19:58</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,12 +6973,12 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:58</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -6987,7 +6987,7 @@
         </is>
       </c>
       <c r="D266" t="n">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>69</v>
+        <v>47</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7028,16 +7028,16 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7053,16 +7053,16 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,21 +7073,21 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>20:24</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>109</v>
+        <v>48</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,21 +7098,21 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>92</v>
+        <v>49</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7128,16 +7128,16 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>20:43</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>110</v>
+        <v>89</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,23 +7148,248 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>69</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>18:35:56</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>20:24</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>109</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>71</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>88</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
           <t>18:53:42</t>
         </is>
       </c>
-      <c r="B273" t="inlineStr">
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>20:43</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>110</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
         <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="C273" t="inlineStr">
+      <c r="C278" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D273" t="n">
-        <v>112</v>
-      </c>
-      <c r="E273" t="inlineStr">
+      <c r="D278" t="n">
+        <v>91</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>101</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>103</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>109</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>116</v>
+      </c>
+      <c r="E282" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7181,7 +7406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7194,14 +7419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:42</t>
+          <t>Última actualización: 19:14:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -8310,7 +8535,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -8324,7 +8549,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>117</v>
+        <v>9</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -8360,23 +8585,73 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>49</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>88</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>18:53:42</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>20:43</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D53" t="n">
         <v>110</v>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8393,7 +8668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8406,14 +8681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:42</t>
+          <t>Última actualización: 19:14:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -9547,23 +9822,73 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>48</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>18:53:42</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D50" t="n">
+      <c r="D51" t="n">
         <v>108</v>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>88</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1869
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E282"/>
+  <dimension ref="A1:E292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:14:20</t>
+          <t>Última actualización: 19:45:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 277</t>
+          <t>Total filas: 287</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4858,7 +4858,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -4873,7 +4873,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -4883,11 +4883,11 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,7 +6173,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -6183,11 +6183,11 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6848,7 +6848,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -6858,11 +6858,11 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6973,12 +6973,12 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>19:58</t>
+          <t>19:57</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -6987,7 +6987,7 @@
         </is>
       </c>
       <c r="D266" t="n">
-        <v>83</v>
+        <v>12</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>18:35:56</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:58</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7048,21 +7048,21 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>69</v>
+        <v>16</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7087,7 +7087,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,12 +7098,12 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -7112,7 +7112,7 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,12 +7148,12 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -7162,7 +7162,7 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,21 +7173,21 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>18:35:56</t>
+          <t>19:14:20</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>20:24</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>109</v>
+        <v>69</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,12 +7198,12 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:24</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -7212,7 +7212,7 @@
         </is>
       </c>
       <c r="D275" t="n">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7228,16 +7228,16 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>20:43</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>110</v>
+        <v>51</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>91</v>
+        <v>56</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7303,16 +7303,16 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,21 +7323,21 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:43</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>109</v>
+        <v>59</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7378,18 +7378,268 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>91</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>19:45:45</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>66</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>101</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>19:45:45</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>71</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>103</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>19:45:45</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>77</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>109</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>19:45:45</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>21:09</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>84</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
           <t>21:10</t>
         </is>
       </c>
-      <c r="C282" t="inlineStr">
+      <c r="C290" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D282" t="n">
+      <c r="D290" t="n">
         <v>116</v>
       </c>
-      <c r="E282" t="inlineStr">
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>19:45:45</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>101</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>19:45:45</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>21:33</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>108</v>
+      </c>
+      <c r="E292" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7406,7 +7656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7419,14 +7669,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:14:20</t>
+          <t>Última actualización: 19:45:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 49</t>
         </is>
       </c>
     </row>
@@ -8560,7 +8810,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -8574,7 +8824,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -8610,12 +8860,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -8624,7 +8874,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>88</v>
+        <v>56</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -8635,23 +8885,48 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>19:14:20</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>88</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>18:53:42</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>20:43</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D53" t="n">
+      <c r="D54" t="n">
         <v>110</v>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8681,7 +8956,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:14:20</t>
+          <t>Última actualización: 19:45:45</t>
         </is>
       </c>
     </row>
@@ -9797,7 +10072,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -9811,7 +10086,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -9847,7 +10122,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -9861,7 +10136,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>108</v>
+        <v>56</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1870
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E292"/>
+  <dimension ref="A1:E298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:45:45</t>
+          <t>Última actualización: 20:01:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 287</t>
+          <t>Total filas: 293</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -858,11 +858,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:49:04</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>06:49:04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:24:16</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>10:24:16</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>18:03:44</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,7 +6173,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>18:03:44</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -6183,11 +6183,11 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,12 +7173,12 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -7187,7 +7187,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>20:24</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,12 +7223,12 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:24</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -7237,7 +7237,7 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,12 +7298,12 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>88</v>
+        <v>56</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,12 +7323,12 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>18:53:42</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>20:43</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -7337,7 +7337,7 @@
         </is>
       </c>
       <c r="D280" t="n">
-        <v>110</v>
+        <v>41</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>18:53:42</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:43</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>59</v>
+        <v>110</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,12 +7373,12 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -7387,7 +7387,7 @@
         </is>
       </c>
       <c r="D282" t="n">
-        <v>91</v>
+        <v>59</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,12 +7423,12 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -7437,7 +7437,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>101</v>
+        <v>66</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7478,16 +7478,16 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7503,16 +7503,16 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>109</v>
+        <v>56</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>21:09</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>84</v>
+        <v>60</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:03</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>101</v>
+        <v>62</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7628,18 +7628,168 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
+          <t>21:09</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>84</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>20:01:01</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>69</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>20:01:01</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>85</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>19:45:45</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
           <t>21:33</t>
         </is>
       </c>
-      <c r="C292" t="inlineStr">
+      <c r="C295" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D292" t="n">
+      <c r="D295" t="n">
         <v>108</v>
       </c>
-      <c r="E292" t="inlineStr">
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>20:01:01</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>93</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>20:01:01</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>95</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>20:01:01</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>105</v>
+      </c>
+      <c r="E298" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7669,7 +7819,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:45:45</t>
+          <t>Última actualización: 20:01:02</t>
         </is>
       </c>
     </row>
@@ -8835,7 +8985,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -8849,7 +8999,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -8885,7 +9035,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -8899,7 +9049,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>88</v>
+        <v>41</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -8956,7 +9106,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:45:45</t>
+          <t>Última actualización: 20:01:02</t>
         </is>
       </c>
     </row>
@@ -10072,7 +10222,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -10086,7 +10236,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -10147,7 +10297,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>19:14:20</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -10161,7 +10311,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>88</v>
+        <v>41</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1871
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E298"/>
+  <dimension ref="A1:E304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:01:02</t>
+          <t>Última actualización: 20:38:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 293</t>
+          <t>Total filas: 299</t>
         </is>
       </c>
     </row>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:35:34</t>
+          <t>16:03:48</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:03:48</t>
+          <t>16:35:34</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>17:26:32</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>17:26:32</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:38:38</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7398,7 +7398,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>20:01:01</t>
+          <t>20:38:38</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -7412,7 +7412,7 @@
         </is>
       </c>
       <c r="D283" t="n">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,7 +7423,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:38:38</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -7437,7 +7437,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>66</v>
+        <v>13</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:38:38</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -7512,7 +7512,7 @@
         </is>
       </c>
       <c r="D287" t="n">
-        <v>71</v>
+        <v>18</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7548,12 +7548,12 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>20:01:01</t>
+          <t>20:38:38</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -7562,7 +7562,7 @@
         </is>
       </c>
       <c r="D289" t="n">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,12 +7598,12 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>20:01:01</t>
+          <t>20:38:38</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -7612,7 +7612,7 @@
         </is>
       </c>
       <c r="D291" t="n">
-        <v>62</v>
+        <v>24</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,21 +7623,21 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:01:01</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>21:09</t>
+          <t>21:03</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,12 +7648,12 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>20:01:01</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>21:09</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -7662,7 +7662,7 @@
         </is>
       </c>
       <c r="D293" t="n">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>20:01:01</t>
+          <t>20:38:38</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,21 +7698,21 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:38:38</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>21:33</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>108</v>
+        <v>48</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,12 +7723,12 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>20:01:01</t>
+          <t>19:45:45</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:33</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -7737,7 +7737,7 @@
         </is>
       </c>
       <c r="D296" t="n">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>20:01:01</t>
+          <t>20:38:38</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>95</v>
+        <v>56</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,23 +7773,173 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
+          <t>20:38:38</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>58</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>20:38:38</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>67</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
           <t>20:01:01</t>
         </is>
       </c>
-      <c r="B298" t="inlineStr">
+      <c r="B300" t="inlineStr">
         <is>
           <t>21:46</t>
         </is>
       </c>
-      <c r="C298" t="inlineStr">
+      <c r="C300" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D298" t="n">
+      <c r="D300" t="n">
         <v>105</v>
       </c>
-      <c r="E298" t="inlineStr">
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>20:38:38</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>22:11</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>93</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>20:38:38</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>22:25</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>107</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>20:38:38</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>115</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>20:38:38</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>22:36</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>118</v>
+      </c>
+      <c r="E304" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7806,7 +7956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7819,14 +7969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:01:02</t>
+          <t>Última actualización: 20:38:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 49</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -9010,7 +9160,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:38:38</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -9024,7 +9174,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -9077,6 +9227,31 @@
         <v>110</v>
       </c>
       <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>20:38:38</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>115</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9093,7 +9268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9106,14 +9281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:01:02</t>
+          <t>Última actualización: 20:38:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 49</t>
         </is>
       </c>
     </row>
@@ -10272,7 +10447,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>19:45:45</t>
+          <t>20:38:38</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -10286,7 +10461,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -10316,6 +10491,56 @@
       <c r="E52" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>20:38:38</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>47</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>20:38:38</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>22:16</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>98</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1872
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-22.xlsx
+++ b/data/horarios-141-2026-03-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E304"/>
+  <dimension ref="A1:E309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:38:38</t>
+          <t>Última actualización: 20:57:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 299</t>
+          <t>Total filas: 304</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>07:40:28</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:40:28</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>76</v>
+        <v>6</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:00:48</t>
+          <t>08:50:24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:50:24</t>
+          <t>08:00:48</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1733,11 +1733,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:23:38</t>
+          <t>12:15:43</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>12:15:43</t>
+          <t>11:23:38</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>13:54:07</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:54:07</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4583,11 +4583,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:16:36</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>14:16:36</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,7 +4873,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14:59:09</t>
+          <t>15:36:22</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -4883,11 +4883,11 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>15:36:22</t>
+          <t>14:59:09</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:58:56</t>
+          <t>16:50:15</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:50:15</t>
+          <t>16:58:56</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>20:01:01</t>
+          <t>20:57:14</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7537,7 +7537,7 @@
         </is>
       </c>
       <c r="D288" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7623,7 +7623,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>20:01:01</t>
+          <t>20:57:14</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7637,7 +7637,7 @@
         </is>
       </c>
       <c r="D292" t="n">
-        <v>62</v>
+        <v>6</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>20:38:38</t>
+          <t>20:57:14</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7687,7 +7687,7 @@
         </is>
       </c>
       <c r="D294" t="n">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>20:38:38</t>
+          <t>20:57:14</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7712,7 +7712,7 @@
         </is>
       </c>
       <c r="D295" t="n">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7748,7 +7748,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>20:38:38</t>
+          <t>20:57:14</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
@@ -7762,7 +7762,7 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>20:38:38</t>
+          <t>20:57:14</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>67</v>
+        <v>43</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,12 +7823,12 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>20:01:01</t>
+          <t>20:38:38</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>21:46</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -7837,7 +7837,7 @@
         </is>
       </c>
       <c r="D300" t="n">
-        <v>105</v>
+        <v>67</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,21 +7848,21 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>20:38:38</t>
+          <t>20:57:14</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>22:11</t>
+          <t>21:46</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>93</v>
+        <v>49</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7873,21 +7873,21 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>20:38:38</t>
+          <t>20:57:14</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>22:25</t>
+          <t>22:04</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>107</v>
+        <v>67</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7898,21 +7898,21 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>20:38:38</t>
+          <t>20:57:14</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>22:33</t>
+          <t>22:11</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>115</v>
+        <v>74</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7928,18 +7928,143 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
+          <t>22:25</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>107</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>20:57:14</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>93</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>20:38:38</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>115</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>20:57:14</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>22:34</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>97</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>20:57:14</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
           <t>22:36</t>
         </is>
       </c>
-      <c r="C304" t="inlineStr">
+      <c r="C308" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D304" t="n">
-        <v>118</v>
-      </c>
-      <c r="E304" t="inlineStr">
+      <c r="D308" t="n">
+        <v>99</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>20:57:14</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>22:44</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>107</v>
+      </c>
+      <c r="E309" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7956,7 +8081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7969,14 +8094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:38:38</t>
+          <t>Última actualización: 20:57:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -9252,6 +9377,31 @@
         <v>115</v>
       </c>
       <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>20:57:14</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>22:34</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>97</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9268,7 +9418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9281,14 +9431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:38:38</t>
+          <t>Última actualización: 20:57:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 49</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -10522,23 +10672,48 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>20:38:38</t>
+          <t>20:57:14</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
+          <t>21:27</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>30</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>20:57:14</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
           <t>22:16</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D54" t="n">
-        <v>98</v>
-      </c>
-      <c r="E54" t="inlineStr">
+      <c r="D55" t="n">
+        <v>79</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>